<commit_message>
feat: complete safety inspection and rectification workflow
</commit_message>
<xml_diff>
--- a/data/规则化数据库/高处作业结构化规则数据库.xlsx
+++ b/data/规则化数据库/高处作业结构化规则数据库.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则库" sheetId="1" r:id="R9fc776dfe5d946cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计摘要" sheetId="2" r:id="R5917d523b7b04b12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规范来源" sheetId="3" r:id="R913a97e1aec94325"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="Rb4173cf82d724d7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="5" r:id="Rd292889af4504dd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规则库" sheetId="1" r:id="R3bdcee0fddd94b8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计摘要" sheetId="2" r:id="R86200a5c70f04994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规范来源" sheetId="3" r:id="Rc1ed061b7e39480a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="4" r:id="R3ccc698f2af34ac4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="5" r:id="R26cdf42c47ec4c82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -876,7 +876,7 @@
         <x:v>GZ-003</x:v>
       </x:c>
       <x:c r="B7" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C7" s="35" t="str">
         <x:v>高处作业综合管理</x:v>
@@ -1691,7 +1691,7 @@
         <x:v>作业准备与过程管理</x:v>
       </x:c>
       <x:c r="E20" s="35" t="str">
-        <x:v>在雨、霜、雾、雪等天气进行高处作业时</x:v>
+        <x:v>露天高处作业施工期间遇雨、霜、雾、雪等天气，或上述天气后恢复作业时</x:v>
       </x:c>
       <x:c r="F20" s="35" t="str">
         <x:v>在雨、霜、雾、雪等天气进行高处作业时，应采取防滑、防冻和防雷措施，并应及时清除作业面上的水、冰、雪、霜</x:v>
@@ -1753,7 +1753,7 @@
         <x:v>作业准备与过程管理</x:v>
       </x:c>
       <x:c r="E21" s="35" t="str">
-        <x:v>当遇有6级及以上强风、浓雾、沙尘暴等恶劣气候</x:v>
+        <x:v>露天攀登或悬空高处作业遇6级及以上强风、浓雾、沙尘暴等恶劣气候时</x:v>
       </x:c>
       <x:c r="F21" s="35" t="str">
         <x:v>当遇有6级及以上强风、浓雾、沙尘暴等恶劣气候，不得进行露天攀登与悬空高处作业</x:v>
@@ -1815,7 +1815,7 @@
         <x:v>作业准备与过程管理</x:v>
       </x:c>
       <x:c r="E22" s="35" t="str">
-        <x:v>雨雪天气后</x:v>
+        <x:v>雨雪天气后恢复高处作业时</x:v>
       </x:c>
       <x:c r="F22" s="35" t="str">
         <x:v>雨雪天气后，应对高处作业安全设施进行检查，当发现有松动、变形、损坏或脱落等现象时，应立即修理完善，维修合格后方可使用</x:v>
@@ -6270,7 +6270,7 @@
         <x:v>XK-007</x:v>
       </x:c>
       <x:c r="B94" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C94" s="35" t="str">
         <x:v>悬空作业</x:v>
@@ -11859,7 +11859,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E184" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含脚手架搭设工序时</x:v>
       </x:c>
       <x:c r="F184" s="35" t="str">
         <x:v>脚手架应按顺序搭设，并应符合下列规定：落地作业脚手架、悬挑脚手架的搭设应与主体结构工程施工同步，一次搭设高度不应超过最上层连墙件2步，且自由高度不应大于4m</x:v>
@@ -11921,7 +11921,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E185" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含脚手架搭设工序时</x:v>
       </x:c>
       <x:c r="F185" s="35" t="str">
         <x:v>剪刀撑、斜撑杆等加固杆件应随架体同步搭设</x:v>
@@ -11983,7 +11983,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E186" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含作业脚手架搭设工序时</x:v>
       </x:c>
       <x:c r="F186" s="35" t="str">
         <x:v>作业脚手架连墙件安装应符合下列规定：连墙件的安装应随作业脚手架搭设同步进行</x:v>
@@ -12107,7 +12107,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E188" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含脚手架搭设工序时</x:v>
       </x:c>
       <x:c r="F188" s="35" t="str">
         <x:v>脚手架安全防护网和防护栏杆等防护设施应随架体搭设同步安装到位</x:v>
@@ -12231,7 +12231,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E190" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>露天脚手架架上作业遇雷雨或6级及以上大风时</x:v>
       </x:c>
       <x:c r="F190" s="35" t="str">
         <x:v>雷雨天气、6级及以上大风天气应停止架上作业</x:v>
@@ -12293,7 +12293,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E191" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>脚手架搭设、拆除或上架作业遇雨、雪、雾、霜天气时</x:v>
       </x:c>
       <x:c r="F191" s="35" t="str">
         <x:v>雨、雪、雾天气应停止脚手架的搭设和拆除作业，雨、雪、霜后上架作业应采取有效的防滑措施，雪天应清除积雪</x:v>
@@ -12355,7 +12355,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E192" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>方案同时采用作业脚手架和支撑脚手架、缆风绳、泵管、卸料平台或大型设备支承件时</x:v>
       </x:c>
       <x:c r="F192" s="35" t="str">
         <x:v>严禁将支撑脚手架、缆风绳、混凝土输送泵管、卸料平台及大型设备的支承件等固定在作业脚手架上</x:v>
@@ -12479,7 +12479,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E194" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>采用支撑脚手架，且进行混凝土浇筑或工程结构件安装等施加荷载工序时</x:v>
       </x:c>
       <x:c r="F194" s="35" t="str">
         <x:v>支撑脚手架在浇筑混凝土、工程结构件安装等施加荷载的过程中，架体下严禁有人</x:v>
@@ -12541,7 +12541,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E195" s="35" t="str">
-        <x:v>在脚手架内进行电焊、气焊和其他动火作业时</x:v>
+        <x:v>方案明确包含脚手架内电焊、气焊、气割或其他动火工序时</x:v>
       </x:c>
       <x:c r="F195" s="35" t="str">
         <x:v>在脚手架内进行电焊、气焊和其他动火作业时，应在动火申请批准后进行作业，并应采取设置接火斗、配置灭火器、移开易燃物等防火措施，同时应设专人监护</x:v>
@@ -12665,7 +12665,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E197" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含脚手架拆除工序时</x:v>
       </x:c>
       <x:c r="F197" s="35" t="str">
         <x:v>架体拆除应按自上而下的顺序按步逐层进行，不应上下同时作业</x:v>
@@ -12727,7 +12727,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E198" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含脚手架拆除工序时</x:v>
       </x:c>
       <x:c r="F198" s="35" t="str">
         <x:v>同层杆件和构配件应按先外后内的顺序拆除</x:v>
@@ -12789,7 +12789,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E199" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含作业脚手架拆除工序时</x:v>
       </x:c>
       <x:c r="F199" s="35" t="str">
         <x:v>作业脚手架连墙件应随架体逐层、同步拆除，不应先将连墙件整层或数层拆除后再拆架体</x:v>
@@ -12851,7 +12851,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E200" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含作业脚手架拆除工序，且拆除中可能形成超过2步的悬臂段时</x:v>
       </x:c>
       <x:c r="F200" s="35" t="str">
         <x:v>作业脚手架拆除作业过程中，当架体悬臂段高度超过2步时，应加设临时拉结</x:v>
@@ -12913,7 +12913,7 @@
         <x:v>脚手架搭设、使用与拆除</x:v>
       </x:c>
       <x:c r="E201" s="35" t="str">
-        <x:v>搭设、使用或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含脚手架拆除及构配件下运工序时</x:v>
       </x:c>
       <x:c r="F201" s="35" t="str">
         <x:v>严禁高空抛掷拆除后的脚手架材料与构配件</x:v>
@@ -15269,7 +15269,7 @@
         <x:v>搭设场地准备</x:v>
       </x:c>
       <x:c r="E239" s="35" t="str">
-        <x:v>搭设、使用、检查或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含脚手架搭设工序时</x:v>
       </x:c>
       <x:c r="F239" s="35" t="str">
         <x:v>脚手架搭设场地应平整、坚实、排水顺畅且不得有积水</x:v>
@@ -15331,7 +15331,7 @@
         <x:v>附着结构核验</x:v>
       </x:c>
       <x:c r="E240" s="35" t="str">
-        <x:v>搭设、使用、检查或拆除施工脚手架时</x:v>
+        <x:v>方案采用与建筑结构附着或拉结的脚手架时</x:v>
       </x:c>
       <x:c r="F240" s="35" t="str">
         <x:v>脚手架附着处的建筑结构混凝土强度应满足安全承载要求</x:v>
@@ -15384,7 +15384,7 @@
         <x:v>JSJ-050</x:v>
       </x:c>
       <x:c r="B241" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C241" s="35" t="str">
         <x:v>脚手架搭设与拆除</x:v>
@@ -15455,7 +15455,7 @@
         <x:v>架体搭设</x:v>
       </x:c>
       <x:c r="E242" s="35" t="str">
-        <x:v>搭设、使用、检查或拆除施工脚手架时</x:v>
+        <x:v>方案采用支撑脚手架并包含搭设工序时</x:v>
       </x:c>
       <x:c r="F242" s="35" t="str">
         <x:v>支撑脚手架应逐排、逐层进行搭设</x:v>
@@ -15508,7 +15508,7 @@
         <x:v>JSJ-052</x:v>
       </x:c>
       <x:c r="B243" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C243" s="35" t="str">
         <x:v>脚手架搭设与拆除</x:v>
@@ -15579,7 +15579,7 @@
         <x:v>架体搭设</x:v>
       </x:c>
       <x:c r="E244" s="35" t="str">
-        <x:v>搭设、使用、检查或拆除施工脚手架时</x:v>
+        <x:v>方案采用构件组装类脚手架并包含搭设工序时</x:v>
       </x:c>
       <x:c r="F244" s="35" t="str">
         <x:v>构件组装类脚手架应自一端向另一端延伸、自下而上按步架设，并逐层改变搭设方向</x:v>
@@ -15641,7 +15641,7 @@
         <x:v>架体搭设</x:v>
       </x:c>
       <x:c r="E245" s="35" t="str">
-        <x:v>搭设、使用、检查或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含脚手架搭设工序时</x:v>
       </x:c>
       <x:c r="F245" s="35" t="str">
         <x:v>每搭设完一步架体后，应校正立杆间距、步距、垂直度及水平杆水平度</x:v>
@@ -15694,7 +15694,7 @@
         <x:v>JSJ-055</x:v>
       </x:c>
       <x:c r="B246" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C246" s="35" t="str">
         <x:v>脚手架搭设与拆除</x:v>
@@ -15765,7 +15765,7 @@
         <x:v>连墙件安装</x:v>
       </x:c>
       <x:c r="E247" s="35" t="str">
-        <x:v>搭设、使用、检查或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含作业脚手架搭设工序，且操作层可能高出相邻连墙件2个步距及以上时</x:v>
       </x:c>
       <x:c r="F247" s="35" t="str">
         <x:v>操作层高出相邻连墙件2个步距及以上时，在上层连墙件安装完毕前必须采取临时拉结措施</x:v>
@@ -15880,7 +15880,7 @@
         <x:v>JSJ-058</x:v>
       </x:c>
       <x:c r="B249" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C249" s="35" t="str">
         <x:v>脚手架搭设与拆除</x:v>
@@ -15942,7 +15942,7 @@
         <x:v>JSJ-059</x:v>
       </x:c>
       <x:c r="B250" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C250" s="35" t="str">
         <x:v>脚手架搭设与拆除</x:v>
@@ -16066,7 +16066,7 @@
         <x:v>JSJ-061</x:v>
       </x:c>
       <x:c r="B252" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C252" s="35" t="str">
         <x:v>脚手架搭设与拆除</x:v>
@@ -16137,7 +16137,7 @@
         <x:v>构配件拆运</x:v>
       </x:c>
       <x:c r="E253" s="35" t="str">
-        <x:v>搭设、使用、检查或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含脚手架拆除及构配件下运工序时</x:v>
       </x:c>
       <x:c r="F253" s="35" t="str">
         <x:v>脚手架拆除作业不得采用重锤击打或撬别</x:v>
@@ -16190,7 +16190,7 @@
         <x:v>JSJ-063</x:v>
       </x:c>
       <x:c r="B254" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C254" s="35" t="str">
         <x:v>脚手架搭设与拆除</x:v>
@@ -16261,7 +16261,7 @@
         <x:v>完工验收</x:v>
       </x:c>
       <x:c r="E255" s="35" t="str">
-        <x:v>搭设、使用、检查或拆除施工脚手架时</x:v>
+        <x:v>方案明确包含脚手架搭设完成并投入使用时</x:v>
       </x:c>
       <x:c r="F255" s="35" t="str">
         <x:v>脚手架搭设完工后应进行验收，验收合格后方可使用</x:v>
@@ -17182,7 +17182,7 @@
         <x:v>MQ-015</x:v>
       </x:c>
       <x:c r="B270" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C270" s="35" t="str">
         <x:v>建筑幕墙设计</x:v>
@@ -17368,7 +17368,7 @@
         <x:v>MQ-018</x:v>
       </x:c>
       <x:c r="B273" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C273" s="35" t="str">
         <x:v>建筑幕墙设计</x:v>
@@ -18112,7 +18112,7 @@
         <x:v>MQ-030</x:v>
       </x:c>
       <x:c r="B285" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C285" s="35" t="str">
         <x:v>建筑幕墙材料</x:v>
@@ -18670,7 +18670,7 @@
         <x:v>MQ-039</x:v>
       </x:c>
       <x:c r="B294" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C294" s="35" t="str">
         <x:v>玻璃幕墙</x:v>
@@ -18794,7 +18794,7 @@
         <x:v>MQ-041</x:v>
       </x:c>
       <x:c r="B296" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C296" s="35" t="str">
         <x:v>玻璃幕墙</x:v>
@@ -18856,7 +18856,7 @@
         <x:v>MQ-042</x:v>
       </x:c>
       <x:c r="B297" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C297" s="35" t="str">
         <x:v>玻璃幕墙</x:v>
@@ -19228,7 +19228,7 @@
         <x:v>MQ-048</x:v>
       </x:c>
       <x:c r="B303" s="41" t="str">
-        <x:v>启用</x:v>
+        <x:v>待核验</x:v>
       </x:c>
       <x:c r="C303" s="35" t="str">
         <x:v>玻璃幕墙</x:v>
@@ -19489,7 +19489,7 @@
       </x:c>
       <x:c r="F5" s="72" t="n">
         <x:f>COUNTIF('规则库'!$B$5:$B$305,"启用")</x:f>
-        <x:v>301</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="G5" s="72"/>
       <x:c r="H5" s="76"/>

</xml_diff>